<commit_message>
Updated the stucture of data excel
</commit_message>
<xml_diff>
--- a/26fall renting.xlsx
+++ b/26fall renting.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\博士\租房\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E030E39-DB13-4396-8EFB-B9D3C7B7120C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DB96B3-E5BE-4023-9579-7DFF98B82942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3291,7 +3291,7 @@
   <cols>
     <col min="1" max="1" width="19.08203125" style="2" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" style="2" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="6.33203125" style="2" customWidth="1"/>
     <col min="4" max="4" width="6.5" style="2" customWidth="1"/>
     <col min="5" max="5" width="6.33203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="5.1640625" style="2" customWidth="1"/>

</xml_diff>